<commit_message>
v6.14.0: STATUS + CAPABILITY-DISCOVERY skills, Status Card (ADR-013)
</commit_message>
<xml_diff>
--- a/core/VCH_HarnessCore.xlsx
+++ b/core/VCH_HarnessCore.xlsx
@@ -383,7 +383,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verifiable Copilot Harness Core v6.13.0</t>
+          <t>Verifiable Copilot Harness Core v6.14.0</t>
         </is>
       </c>
     </row>
@@ -395,7 +395,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Verifiable Copilot Harness Core v6.13.0 (behavior-only)</t>
+          <t>Verifiable Copilot Harness Core v6.14.0 (behavior-only)</t>
         </is>
       </c>
     </row>
@@ -419,7 +419,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
     </row>
@@ -431,7 +431,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>43</t>
         </is>
       </c>
     </row>
@@ -443,7 +443,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Skills 1-33 INDEPENDENT_READ_BACK from v6.8.1; +6 by ADR-005; hardened by ADR-007; PROJECT-GUIDE + lifecycle state by ADR-008; FOCUS-MODE by ADR-009; version-independent filenames by ADR-010; one-active-workbook modes by ADR-011; __ROUTING_ORACLE behavioral regression (out-of-bootstrap) by ADR-012.</t>
+          <t>Skills 1-33 INDEPENDENT_READ_BACK from v6.8.1; +6 by ADR-005; hardened by ADR-007; PROJECT-GUIDE + lifecycle state by ADR-008; FOCUS-MODE by ADR-009; version-independent filenames by ADR-010; one-active-workbook modes by ADR-011; __ROUTING_ORACLE behavioral regression (out-of-bootstrap) by ADR-012. v6.14.0 adds STATUS and CAPABILITY-DISCOVERY plus the Status Card (43 skills) by ADR-013.</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Canonical version = v6.13.0; canonical NONE token = NONE; enum values are field-scoped; oracle, routing oracle, ADR and glossary cells are text-only.</t>
+          <t>Canonical version = v6.14.0; canonical NONE token = NONE; enum values are field-scoped; oracle, routing oracle, ADR and glossary cells are text-only.</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FROZEN ROUTING ORACLE v6.13.0 (out-of-bootstrap; L2 routing + L3 adversarial)</t>
+          <t>FROZEN ROUTING ORACLE v6.14.0 (out-of-bootstrap; L2 routing + L3 adversarial)</t>
         </is>
       </c>
     </row>
@@ -3382,6 +3382,162 @@
       <c r="J54" s="3" t="inlineStr">
         <is>
           <t>read once; Active_Behavior_Source_Count=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>RT-053</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>EXACT</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>literal_trigger</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>read-only status card, no writes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>RT-054</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>EXACT</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>what can you do</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>literal_trigger</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>CAPABILITY-DISCOVERY</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>context-aware discovery, conservative</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>RT-055</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>ALT</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>where are we</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>alt_trigger_atom</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>alt of status / where are we / current status</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3418,7 +3574,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SKILL CATALOGUE v6.13.0</t>
+          <t>SKILL CATALOGUE v6.14.0</t>
         </is>
       </c>
     </row>
@@ -3542,7 +3698,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -3612,7 +3768,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -3684,7 +3840,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -3754,7 +3910,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -3824,7 +3980,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -3894,7 +4050,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -3964,7 +4120,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -4034,7 +4190,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -4104,7 +4260,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -4174,7 +4330,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -4244,7 +4400,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -4314,7 +4470,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -4384,7 +4540,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -4454,7 +4610,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -4524,7 +4680,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -4594,7 +4750,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -4664,7 +4820,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -4734,7 +4890,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -4804,7 +4960,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -4874,7 +5030,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -4944,7 +5100,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -5014,7 +5170,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -5084,7 +5240,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -5154,7 +5310,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -5224,7 +5380,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -5294,7 +5450,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -5364,7 +5520,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -5434,7 +5590,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -5504,7 +5660,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -5574,7 +5730,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -5644,7 +5800,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -5714,7 +5870,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -5784,7 +5940,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -5854,7 +6010,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -5924,7 +6080,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -5994,7 +6150,7 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -6064,7 +6220,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -6134,7 +6290,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -6204,7 +6360,7 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -6274,7 +6430,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -6344,7 +6500,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -6414,7 +6570,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -6431,6 +6587,150 @@
         <v>96</v>
       </c>
       <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>status / where are we / current status</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Read-only current status report (Status Card).</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Read __STATE, gate status and evidence-qualified verified items from the active behavior source; output only the Status Card; never write.</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Status Card fields: Mode, Resume (literal Resume_From or none), Gate (PASS, BLOCKED, NOT_TESTED or n/a), Verified (max 3 INDEPENDENT_READ_BACK or TOOL_TRANSACTION_REPORT items), Next (one concrete action). The card is always the last block; only a short VERSION_MISMATCH or WRITE_BLOCKED warning may precede it.</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Read-only; never writes to the workbook.</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Same behavior in FOCUS MODE; no prose around the card.</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>v6.14.0</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>User asks for a quick reliable current-state overview without further work.</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Do not use to change state or continue delivery.</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>CAPABILITY-DISCOVERY</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Capability Discovery</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>what can you do / available skills</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Knowledge</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Context-aware list of skills usable right now.</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Detect workbook mode, open gates, runtime capability and persistence; list only skills allowed now; max 5-6 entries; never the full catalog.</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Output an AVAILABLE NOW block: Mode, High priority (Skill_ID -&gt; shortest trigger and one-line purpose), Also available, Blocked (with reason: gate, mode or capability). Conservative: never suggest skills that would violate current Persistence_Mode, runtime capability or phase gates. In FOCUS MODE shorten further, high priority only.</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Read-only analysis; never writes to the workbook.</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Uses runtime capability only; never stored PASS state.</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>v6.14.0</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>User asks which skills make sense right now, not the full catalog.</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>Do not use for a full catalog listing or when routing to a specific skill is already clear.</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
@@ -6458,7 +6758,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PROJECT.RULES v6.13.0</t>
+          <t>PROJECT.RULES v6.14.0</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6926,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>All components must agree on v6.13.0.</t>
+          <t>All components must agree on v6.14.0.</t>
         </is>
       </c>
     </row>
@@ -6734,7 +7034,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Use v6.13.0 for all harness and skill versions and NONE for an explicit empty canonical alternative. The strings None and none are forbidden as canonical tokens. Artifact_Status=REJECTED and Output_Verification_Status=OUTPUT_REJECTED are distinct field-scoped states.</t>
+          <t>Use v6.14.0 for all harness and skill versions and NONE for an explicit empty canonical alternative. The strings None and none are forbidden as canonical tokens. Artifact_Status=REJECTED and Output_Verification_Status=OUTPUT_REJECTED are distinct field-scoped states.</t>
         </is>
       </c>
     </row>
@@ -6856,7 +7156,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>__STATE v6.13.0</t>
+          <t>__STATE v6.14.0</t>
         </is>
       </c>
     </row>
@@ -6888,7 +7188,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
     </row>
@@ -6912,7 +7212,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7344,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>VCH_HarnessCore.xlsx v6.12.0</t>
+          <t>VCH_HarnessCore.xlsx v6.13.0</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7572,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>VCH_HarnessCore.xlsx v6.12.0; ADR-012</t>
+          <t>VCH_HarnessCore.xlsx v6.13.0; ADR-013</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7658,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>00 Landing v6.13.0</t>
+          <t>00 Landing v6.14.0</t>
         </is>
       </c>
     </row>
@@ -7462,7 +7762,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7985,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FROZEN TEST ORACLE v6.13.0</t>
+          <t>FROZEN TEST ORACLE v6.14.0</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8336,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>43</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -8061,7 +8361,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>00_Skills must have exactly 41 non-empty Skill_ID.</t>
+          <t>00_Skills must have exactly 43 non-empty Skill_ID.</t>
         </is>
       </c>
     </row>
@@ -8083,7 +8383,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -8108,7 +8408,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>All version fields across sheets agree on v6.13.0.</t>
+          <t>All version fields across sheets agree on v6.14.0.</t>
         </is>
       </c>
     </row>
@@ -8130,7 +8430,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>v6.13.0</t>
+          <t>v6.14.0</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -8155,7 +8455,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>All 41 skill rows use canonical v6.13.0.</t>
+          <t>All 43 skill rows use canonical v6.14.0.</t>
         </is>
       </c>
     </row>
@@ -8932,7 +9232,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CANONICAL LISTS v6.13.0</t>
+          <t>CANONICAL LISTS v6.14.0</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10143,7 +10443,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Add __ROUTING_ORACLE behavioral regression sheet (out-of-bootstrap) and bump to v6.13.0</t>
+          <t>Add __ROUTING_ORACLE behavioral regression sheet (out-of-bootstrap) and bump to v6.14.0</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -10163,7 +10463,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Adds one sheet to both HarnessCore and ProjectTemplate; skill count stays 41 (routing oracle is data, not a skill); three ROUTING oracle rows added to __TEST_ORACLE; two glossary terms added (Routing oracle, Behavioral test); Project.Rules gains a ROUTING ORACLE rule; starter, custom instructions and cheatsheet updated to declare the out-of-bootstrap corpus; all components bumped to v6.13.0. ADR-012 supersedes the fixed B32 probe-address assumption in ADR-008; PROBE_CELL resolved by name is authoritative.</t>
+          <t>Adds one sheet to both HarnessCore and ProjectTemplate; skill count stays 41 (routing oracle is data, not a skill); three ROUTING oracle rows added to __TEST_ORACLE; two glossary terms added (Routing oracle, Behavioral test); Project.Rules gains a ROUTING ORACLE rule; starter, custom instructions and cheatsheet updated to declare the out-of-bootstrap corpus; all components bumped to v6.14.0. ADR-012 supersedes the fixed B32 probe-address assumption in ADR-008; PROBE_CELL resolved by name is authoritative.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -10173,7 +10473,59 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Independent reopen of both v6.13.0 workbooks; deterministic structural checks: 41 skills, __ROUTING_ORACLE present and out of bootstrap read-set, 0 unresolved Expected_Skill_ID references, 0 duplicate routing Test_ID, version agreement PASS, probe cell intact. Independent read-back confirms PROBE_CELL resolves to __STATE!B31.</t>
+          <t>Independent reopen of both v6.14.0 workbooks; deterministic structural checks: 41 skills, __ROUTING_ORACLE present and out of bootstrap read-set, 0 unresolved Expected_Skill_ID references, 0 duplicate routing Test_ID, version agreement PASS, probe cell intact. Independent read-back confirms PROBE_CELL resolves to __STATE!B31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ADR-013</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Add STATUS and CAPABILITY-DISCOVERY skills plus a mandatory Status Card (43 skills) and bump to v6.14.0</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>External proposal (Grok) reviewed and adapted: a compact Status Card after key events, a cheap read-only STATUS atom, and a conservative context-aware skill discovery. Czech and diacritic trigger atoms were dropped (character policy), the colliding atom 'what can you do now' was dropped (prefix collision with 'what can you do'), and non-ASCII arrows in templates were replaced with -&gt;.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Adopt as proposed; adopt with trigger and ASCII corrections; reject.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Adopted with corrections: the Status Card formalizes state restatement already required by FOCUS-MODE rule 5 and bootstrap discipline; STATUS is cheap and read-only; CAPABILITY-DISCOVERY never suggests skills violating current gates, persistence or runtime capability. All new trigger atoms are unique, prefix-collision-free ASCII English atoms.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Skill count becomes 43 (oracle, _README and lint updated); routing corpus grows to 55 fixtures; custom instructions and starter gain a STATUS CARD contract; cheatsheet and README updated.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Revert to the v6.13.0 artifacts (release assets VCH_v6.13.0.zip).</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Deterministic scan on reopened v6.14.0 workbooks: 43 skills, trigger duplicates 0, prefix collisions 0, non-ASCII cells 0, routing 55/55 refs resolved, probe B31, version agreement v6.14.0.</t>
         </is>
       </c>
     </row>
@@ -10189,7 +10541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10879,6 +11231,38 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Status card</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory compact status block appended at the very end of replies after key events (bootstrap, guide steps, gates, revision commits, update context, explicit status): Mode, Resume, Gate, Verified (evidence-qualified only), Next.</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>status block</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>prose summary at reply start</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>ADR-013</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
v6.15.0: Allowed_Modes column (ADR-014)
</commit_message>
<xml_diff>
--- a/core/VCH_HarnessCore.xlsx
+++ b/core/VCH_HarnessCore.xlsx
@@ -383,7 +383,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verifiable Copilot Harness Core v6.14.0</t>
+          <t>Verifiable Copilot Harness Core v6.15.0</t>
         </is>
       </c>
     </row>
@@ -395,7 +395,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Verifiable Copilot Harness Core v6.14.0 (behavior-only)</t>
+          <t>Verifiable Copilot Harness Core v6.15.0 (behavior-only)</t>
         </is>
       </c>
     </row>
@@ -419,7 +419,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
     </row>
@@ -443,7 +443,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Skills 1-33 INDEPENDENT_READ_BACK from v6.8.1; +6 by ADR-005; hardened by ADR-007; PROJECT-GUIDE + lifecycle state by ADR-008; FOCUS-MODE by ADR-009; version-independent filenames by ADR-010; one-active-workbook modes by ADR-011; __ROUTING_ORACLE behavioral regression (out-of-bootstrap) by ADR-012. v6.14.0 adds STATUS and CAPABILITY-DISCOVERY plus the Status Card (43 skills) by ADR-013.</t>
+          <t>Skills 1-33 INDEPENDENT_READ_BACK from v6.8.1; +6 by ADR-005; hardened by ADR-007; PROJECT-GUIDE + lifecycle state by ADR-008; FOCUS-MODE by ADR-009; version-independent filenames by ADR-010; one-active-workbook modes by ADR-011; __ROUTING_ORACLE behavioral regression (out-of-bootstrap) by ADR-012. v6.15.0 adds STATUS and CAPABILITY-DISCOVERY plus the Status Card (43 skills) by ADR-013. v6.15.0 adds the Allowed_Modes column by ADR-014.</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Canonical version = v6.14.0; canonical NONE token = NONE; enum values are field-scoped; oracle, routing oracle, ADR and glossary cells are text-only.</t>
+          <t>Canonical version = v6.15.0; canonical NONE token = NONE; enum values are field-scoped; oracle, routing oracle, ADR and glossary cells are text-only.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FROZEN ROUTING ORACLE v6.14.0 (out-of-bootstrap; L2 routing + L3 adversarial)</t>
+          <t>FROZEN ROUTING ORACLE v6.15.0 (out-of-bootstrap; L2 routing + L3 adversarial)</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3574,7 +3574,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SKILL CATALOGUE v6.14.0</t>
+          <t>SKILL CATALOGUE v6.15.0</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -3719,6 +3719,11 @@
           <t>BOOTSTRAP-CHECK, CAPABILITY-ROUTER</t>
         </is>
       </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Allowed_Modes</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.85" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -3768,7 +3773,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -3789,6 +3794,11 @@
       <c r="N4" s="3" t="inlineStr">
         <is>
           <t>BOOTSTRAP-CHECK, CAPABILITY-ROUTER</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3850,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -3861,6 +3871,11 @@
           <t>GRILL-ME</t>
         </is>
       </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="35.1" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -3910,7 +3925,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -3931,6 +3946,11 @@
           <t>SHAPING</t>
         </is>
       </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.85" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -3980,7 +4000,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -4001,6 +4021,11 @@
           <t>SHAPING</t>
         </is>
       </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="23.85" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -4050,7 +4075,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -4071,6 +4096,11 @@
           <t>SHAPING</t>
         </is>
       </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="23.85" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -4120,7 +4150,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -4141,6 +4171,11 @@
           <t>UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="23.85" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -4190,7 +4225,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -4211,6 +4246,11 @@
           <t>WRITING-PITCH</t>
         </is>
       </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="23.85" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -4260,7 +4300,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -4281,6 +4321,11 @@
           <t>PROOF</t>
         </is>
       </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4330,7 +4375,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -4351,6 +4396,11 @@
           <t>WRITING-PLANS</t>
         </is>
       </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="23.85" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -4400,7 +4450,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -4421,6 +4471,11 @@
           <t>PLAN-DEEPENING</t>
         </is>
       </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="23.85" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -4470,7 +4525,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -4491,6 +4546,11 @@
           <t>VERIFICATION-CHECKLIST</t>
         </is>
       </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="23.85" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -4540,7 +4600,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -4561,6 +4621,11 @@
           <t>VERIFICATION-CHECKLIST</t>
         </is>
       </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="23.85" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4610,7 +4675,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -4631,6 +4696,11 @@
           <t>UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="23.85" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -4680,7 +4750,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -4701,6 +4771,11 @@
           <t>SCRUB</t>
         </is>
       </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="23.85" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -4750,7 +4825,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -4771,6 +4846,11 @@
           <t>COMPOUND</t>
         </is>
       </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="23.85" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -4820,7 +4900,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -4841,6 +4921,11 @@
           <t>HARDEN-SCRIPT</t>
         </is>
       </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="23.85" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -4890,7 +4975,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -4911,6 +4996,11 @@
           <t>SHAPING</t>
         </is>
       </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="23.85" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -4960,7 +5050,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -4981,6 +5071,11 @@
           <t>SHAPING</t>
         </is>
       </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="23.85" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -5030,7 +5125,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -5051,6 +5146,11 @@
           <t>VERIFICATION-CHECKLIST</t>
         </is>
       </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="23.85" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -5100,7 +5200,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -5121,6 +5221,11 @@
           <t>COMPOUND</t>
         </is>
       </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23.85" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -5170,7 +5275,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -5191,6 +5296,11 @@
           <t>BUILD-TOOL</t>
         </is>
       </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="23.85" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -5240,7 +5350,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -5261,6 +5371,11 @@
           <t>PROOF</t>
         </is>
       </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.85" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -5310,7 +5425,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -5331,6 +5446,11 @@
           <t>HARDEN-SCRIPT</t>
         </is>
       </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="23.85" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -5380,7 +5500,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -5401,6 +5521,11 @@
           <t>SCRUB</t>
         </is>
       </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="23.85" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -5450,7 +5575,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -5471,6 +5596,11 @@
           <t>WRITING-PLANS</t>
         </is>
       </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="23.85" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -5520,7 +5650,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -5541,6 +5671,11 @@
           <t>UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="23.85" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -5590,7 +5725,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -5611,6 +5746,11 @@
           <t>PROOF</t>
         </is>
       </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="23.85" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -5660,7 +5800,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -5681,6 +5821,11 @@
           <t>CAPABILITY-ROUTER</t>
         </is>
       </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="35.1" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
@@ -5730,7 +5875,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -5751,6 +5896,11 @@
           <t>WRITING-PLANS</t>
         </is>
       </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>TEMPLATE, PROJECT-CREATION, MIGRATION</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="23.85" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
@@ -5800,7 +5950,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -5821,6 +5971,11 @@
           <t>UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="35.1" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
@@ -5870,7 +6025,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -5891,6 +6046,11 @@
           <t>PROJECT-FORK, ACTIVATE-PRECOPIED-REVISION, INPLACE-CHECKPOINT</t>
         </is>
       </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="35.1" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
@@ -5940,7 +6100,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -5961,6 +6121,11 @@
           <t>UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="35.1" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
@@ -6010,7 +6175,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -6031,6 +6196,11 @@
           <t>UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="35.1" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -6080,7 +6250,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -6101,6 +6271,11 @@
           <t>TRIAGE</t>
         </is>
       </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="23.85" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
@@ -6150,7 +6325,7 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -6171,6 +6346,11 @@
           <t>VERIFICATION-CHECKLIST</t>
         </is>
       </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="35.1" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
@@ -6220,7 +6400,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -6241,6 +6421,11 @@
           <t>COMPARE</t>
         </is>
       </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="23.85" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -6290,7 +6475,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -6311,6 +6496,11 @@
           <t>COMPOUND</t>
         </is>
       </c>
+      <c r="O40" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="23.85" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -6360,7 +6550,7 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -6381,6 +6571,11 @@
           <t>HARDEN-SCRIPT</t>
         </is>
       </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="90.95" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
@@ -6430,7 +6625,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -6451,6 +6646,11 @@
           <t>WRITING-PLANS</t>
         </is>
       </c>
+      <c r="O42" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="68.65000000000001" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -6500,7 +6700,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -6521,6 +6721,11 @@
           <t>PROJECT-FORK, CAPABILITY-ROUTER, GRILL-ME, IDEATE, SHAPING, WRITING-PLANS, PLAN-DEEPENING, SYSTEMATIC-DEBUGGING, BUILD-TOOL, HARDEN-SCRIPT, VERIFICATION-CHECKLIST, SCRUB, COMPOUND, DECISION-DRIFT-CHECK, UPDATE-CONTEXT</t>
         </is>
       </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT, PROJECT-CREATION, MIGRATION</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -6570,7 +6775,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -6591,6 +6796,11 @@
           <t>NONE</t>
         </is>
       </c>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -6640,7 +6850,7 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -6661,6 +6871,11 @@
       <c r="N45" s="3" t="inlineStr">
         <is>
           <t>NONE</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6917,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>Read-only analysis; never writes to the workbook.</t>
+          <t>Output an AVAILABLE NOW block: Mode, High priority (Skill_ID -&gt; shortest trigger and one-line purpose), Also available, Blocked (with reason: gate, mode or capability). Filter first by the Allowed_Modes column against the current workbook mode, then by gates and runtime capability. Conservative: never suggest skills that would violate current Persistence_Mode, runtime capability or phase gates. In FOCUS MODE shorten further, high priority only.</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -6712,7 +6927,7 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
@@ -6733,6 +6948,11 @@
       <c r="N46" s="3" t="inlineStr">
         <is>
           <t>NONE</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6758,7 +6978,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PROJECT.RULES v6.14.0</t>
+          <t>PROJECT.RULES v6.15.0</t>
         </is>
       </c>
     </row>
@@ -6926,7 +7146,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>All components must agree on v6.14.0.</t>
+          <t>All components must agree on v6.15.0.</t>
         </is>
       </c>
     </row>
@@ -7034,7 +7254,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Use v6.14.0 for all harness and skill versions and NONE for an explicit empty canonical alternative. The strings None and none are forbidden as canonical tokens. Artifact_Status=REJECTED and Output_Verification_Status=OUTPUT_REJECTED are distinct field-scoped states.</t>
+          <t>Use v6.15.0 for all harness and skill versions and NONE for an explicit empty canonical alternative. The strings None and none are forbidden as canonical tokens. Artifact_Status=REJECTED and Output_Verification_Status=OUTPUT_REJECTED are distinct field-scoped states.</t>
         </is>
       </c>
     </row>
@@ -7131,6 +7351,18 @@
       <c r="B32" s="3" t="inlineStr">
         <is>
           <t>__ROUTING_ORACLE is a frozen behavioral regression corpus (L2 routing, L3 adversarial). It is NOT part of the bootstrap read-set and must not be read on load vch. Run it only on explicit request or before promoting a catalogue change. Every Expected_Skill_ID must be NONE or an existing Skill_ID. Model routing runs are behavioral tests; harness_lint validates only structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>ALLOWED MODES</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>00_Skills.Allowed_Modes declares in which workbook modes a skill may run: ALL or a comma-space separated subset of HARNESS, TEMPLATE, PROJECT-CREATION, PROJECT, MIGRATION. Routing and CAPABILITY-DISCOVERY must not propose a skill outside its Allowed_Modes.</t>
         </is>
       </c>
     </row>
@@ -7156,7 +7388,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>__STATE v6.14.0</t>
+          <t>__STATE v6.15.0</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7420,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
     </row>
@@ -7212,7 +7444,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7576,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>VCH_HarnessCore.xlsx v6.13.0</t>
+          <t>VCH_HarnessCore.xlsx v6.14.0</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7804,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>VCH_HarnessCore.xlsx v6.13.0; ADR-013</t>
+          <t>VCH_HarnessCore.xlsx v6.14.0; ADR-014</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7890,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>00 Landing v6.14.0</t>
+          <t>00 Landing v6.15.0</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7994,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
     </row>
@@ -7970,7 +8202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7985,7 +8217,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FROZEN TEST ORACLE v6.14.0</t>
+          <t>FROZEN TEST ORACLE v6.15.0</t>
         </is>
       </c>
     </row>
@@ -8383,7 +8615,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -8408,7 +8640,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>All version fields across sheets agree on v6.14.0.</t>
+          <t>All version fields across sheets agree on v6.15.0.</t>
         </is>
       </c>
     </row>
@@ -8430,7 +8662,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>v6.14.0</t>
+          <t>v6.15.0</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -8455,7 +8687,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>All 43 skill rows use canonical v6.14.0.</t>
+          <t>All 43 skill rows use canonical v6.15.0.</t>
         </is>
       </c>
     </row>
@@ -9208,6 +9440,53 @@
       <c r="I27" s="3" t="inlineStr">
         <is>
           <t>All __ROUTING_ORACLE Test_ID values are unique. Structural check only; behavioral routing requires an isolated routing run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>NORMALIZATION</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Allowed_Modes_Valid</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>DETERMINISTIC_SCAN</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Every 00_Skills.Allowed_Modes value is ALL or a comma-space separated subset of HARNESS, TEMPLATE, PROJECT-CREATION, PROJECT, MIGRATION.</t>
         </is>
       </c>
     </row>
@@ -9232,7 +9511,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CANONICAL LISTS v6.14.0</t>
+          <t>CANONICAL LISTS v6.15.0</t>
         </is>
       </c>
     </row>
@@ -9935,7 +10214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10443,7 +10722,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Add __ROUTING_ORACLE behavioral regression sheet (out-of-bootstrap) and bump to v6.14.0</t>
+          <t>Add __ROUTING_ORACLE behavioral regression sheet (out-of-bootstrap) and bump to v6.15.0</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -10463,7 +10742,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Adds one sheet to both HarnessCore and ProjectTemplate; skill count stays 41 (routing oracle is data, not a skill); three ROUTING oracle rows added to __TEST_ORACLE; two glossary terms added (Routing oracle, Behavioral test); Project.Rules gains a ROUTING ORACLE rule; starter, custom instructions and cheatsheet updated to declare the out-of-bootstrap corpus; all components bumped to v6.14.0. ADR-012 supersedes the fixed B32 probe-address assumption in ADR-008; PROBE_CELL resolved by name is authoritative.</t>
+          <t>Adds one sheet to both HarnessCore and ProjectTemplate; skill count stays 41 (routing oracle is data, not a skill); three ROUTING oracle rows added to __TEST_ORACLE; two glossary terms added (Routing oracle, Behavioral test); Project.Rules gains a ROUTING ORACLE rule; starter, custom instructions and cheatsheet updated to declare the out-of-bootstrap corpus; all components bumped to v6.15.0. ADR-012 supersedes the fixed B32 probe-address assumption in ADR-008; PROBE_CELL resolved by name is authoritative.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -10473,7 +10752,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Independent reopen of both v6.14.0 workbooks; deterministic structural checks: 41 skills, __ROUTING_ORACLE present and out of bootstrap read-set, 0 unresolved Expected_Skill_ID references, 0 duplicate routing Test_ID, version agreement PASS, probe cell intact. Independent read-back confirms PROBE_CELL resolves to __STATE!B31.</t>
+          <t>Independent reopen of both v6.15.0 workbooks; deterministic structural checks: 41 skills, __ROUTING_ORACLE present and out of bootstrap read-set, 0 unresolved Expected_Skill_ID references, 0 duplicate routing Test_ID, version agreement PASS, probe cell intact. Independent read-back confirms PROBE_CELL resolves to __STATE!B31.</t>
         </is>
       </c>
     </row>
@@ -10495,7 +10774,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Add STATUS and CAPABILITY-DISCOVERY skills plus a mandatory Status Card (43 skills) and bump to v6.14.0</t>
+          <t>Add STATUS and CAPABILITY-DISCOVERY skills plus a mandatory Status Card (43 skills) and bump to v6.15.0</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -10525,7 +10804,59 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Deterministic scan on reopened v6.14.0 workbooks: 43 skills, trigger duplicates 0, prefix collisions 0, non-ASCII cells 0, routing 55/55 refs resolved, probe B31, version agreement v6.14.0.</t>
+          <t>Deterministic scan on reopened v6.15.0 workbooks: 43 skills, trigger duplicates 0, prefix collisions 0, non-ASCII cells 0, routing 55/55 refs resolved, probe B31, version agreement v6.15.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Add Allowed_Modes column to 00_Skills for deterministic mode-based skill filtering and bump to v6.15.0</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>CAPABILITY-DISCOVERY (ADR-013) judged mode eligibility from Use_When prose, which is soft. A machine-readable allowlist makes mode filtering deterministic and lint-enforceable.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Prose-only filtering; Allowed_Modes column with ALL or an explicit mode subset.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>A catalog column is declarative, validated by the deterministic lint, and keeps CAPABILITY-DISCOVERY conservative by construction: persistence skills are PROJECT-only, forking is TEMPLATE, PROJECT-CREATION and MIGRATION only, orchestration stays with project modes.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>00_Skills gains column Allowed_Modes (ALL or comma-space separated subset of HARNESS, TEMPLATE, PROJECT-CREATION, PROJECT, MIGRATION); Project.Rules gains ALLOWED MODES; oracle gains Allowed_Modes_Valid DETERMINISTIC_SCAN; harness_lint validates values; CAPABILITY-DISCOVERY behavior now references the column.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Revert to the v6.14.0 artifacts (release assets VCH_v6.14.0.zip).</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Deterministic scan on reopened v6.15.0 workbooks: 43 skills, Allowed_Modes 43/43 valid, trigger duplicates 0, prefix collisions 0, non-ASCII 0, routing 55/55 refs resolved, probe B31, version agreement v6.15.0.</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11263,6 +11594,38 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Allowed modes</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>00_Skills.Allowed_Modes value declaring in which workbook modes a skill may run: ALL or a comma-space separated subset of HARNESS, TEMPLATE, PROJECT-CREATION, PROJECT, MIGRATION. Routing and CAPABILITY-DISCOVERY must not propose a skill outside its Allowed_Modes.</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>mode allowlist</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>soft prose-based filtering</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
v0.7.1: embed starter as _STARTER sheet (ADR-019)
One attached file remains: the core workbook. The starter text is now a
generated _STARTER sheet (position 2, after _README); copilot/copilotstart.txt
stays in the repo as the source of truth (sheet is generated, never edited).

- core: _STARTER sheet (94 lines), ADR-019 (Proposed), oracle row
  STARTER/Starter_Sheet_Present, glossary term, version bump 0.7.0 -> 0.7.1
- lint: _STARTER in RequiredSheets + ASCII scan, new Test-StarterSheet
  (sheet vs file, non-empty lines, ordinal) - pending first Windows COM run
- copilot texts: read-set starts with _STARTER, attach only the workbook
- verify: 35/35 PASS, FORK_GATE simulation PASS
- accept_adrs.py: ADR-016..019, v0.7.1 messages
- docs: README, cheatsheet, RUNBOOK_gates, WIN_GUIDE, RELEASING, plan;
  release_notes_v0.7.1.md; manifest regenerated
</commit_message>
<xml_diff>
--- a/core/VCH_HarnessCore.xlsx
+++ b/core/VCH_HarnessCore.xlsx
@@ -7,16 +7,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Skills" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project.Rules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__STATE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Landing" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__TEST_ORACLE" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__ADR" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__GLOSSARY" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__ROUTING_ORACLE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__DELIVERY_SCHEMA" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_STARTER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Skills" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project.Rules" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__STATE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Landing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__TEST_ORACLE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__ADR" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__GLOSSARY" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__ROUTING_ORACLE" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__DELIVERY_SCHEMA" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="PROBE_CELL">__STATE!$B$31</definedName>
@@ -387,7 +388,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verifiable Copilot Harness Core v0.7.0</t>
+          <t>Verifiable Copilot Harness Core v0.7.1</t>
         </is>
       </c>
     </row>
@@ -399,7 +400,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Verifiable Copilot Harness Core v0.7.0 (single behavior kernel)</t>
+          <t>Verifiable Copilot Harness Core v0.7.1 (single behavior kernel)</t>
         </is>
       </c>
     </row>
@@ -423,7 +424,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
     </row>
@@ -519,7 +520,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Canonical version = v0.7.0; canonical NONE token = NONE; enum values are field-scoped; oracle, routing oracle, ADR and glossary cells are text-only.</t>
+          <t>Canonical version = v0.7.1; canonical NONE token = NONE; enum values are field-scoped; oracle, routing oracle, ADR and glossary cells are text-only.</t>
         </is>
       </c>
     </row>
@@ -531,7 +532,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Project.Rules, 00_Landing, __STATE, 00_Skills, __TEST_ORACLE, __ADR, __GLOSSARY. __ROUTING_ORACLE and __DELIVERY_SCHEMA are NOT in the bootstrap read-set; PROJECT-FORK reads __DELIVERY_SCHEMA at fork.</t>
+          <t>_STARTER, Project.Rules, 00_Landing, __STATE, 00_Skills, __TEST_ORACLE, __ADR, __GLOSSARY. __ROUTING_ORACLE and __DELIVERY_SCHEMA are NOT in the bootstrap read-set; PROJECT-FORK reads __DELIVERY_SCHEMA at fork.</t>
         </is>
       </c>
     </row>
@@ -554,6 +555,804 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.5" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROJECT GLOSSARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Aliases</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Do_Not_Use</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Host mode</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Workbook interaction context independent from capability.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>OPEN_WORKBOOK</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>write capability</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>ADR-004</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Precopied artifact</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>User-created canonical next revision verified before activation.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Save a Copy target</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>storage suffix copy</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ADR-004</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Logical checkpoint</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Verified in-place state change with no new physical artifact.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>native revision</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>physical revision</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>ADR-004</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="23.9" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Trigger delimiter</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ASCII sequence " / " separating alternative literal triggers only in 00_Skills.Trigger.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>slash-delimited aliases</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>global slash splitting</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="23.9" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Chain delimiter</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ASCII sequence ", " separating Skill_ID values only in 00_Skills.May_Chain_To.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>comma-delimited chain</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>global comma splitting</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Field-scoped enum</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Canonical enum value interpreted together with its field name.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Field=Value</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>unqualified status token</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="23.9" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Output rejected</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Output verification state OUTPUT_REJECTED; distinct from Artifact_Status=REJECTED.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>OUTPUT_REJECTED</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>artifact rejected</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="23.9" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Artifact rejected</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Artifact lifecycle state REJECTED; distinct from Output_Verification_Status=OUTPUT_REJECTED.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>output rejected</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Canonical NONE</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Explicit empty canonical alternative represented by ASCII token NONE.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>None / none</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="35.15" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Sovereign rules</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Safety rules that no lower authority layer may weaken: SCRUB, FROZEN ORACLE, EVIDENCE, NO CAPABILITY INHERITANCE, CHARACTER POLICY.</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>authority layer 0</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>overridable safety</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>ADR-007</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="23.9" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Version migration</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Controlled port of an older-version workbook into a new revision forked from the current kernel after a VERSION_MISMATCH report.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>kernel upgrade</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>silent rewrite</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>ADR-007</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="35.15" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Probe cell</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Value cell of the __WRITE_PROBE field in __STATE, exposed as named range PROBE_CELL (currently __STATE!B31); the only legal direct-edit probe target, always resolved by name.</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>PROBE_CELL</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>fixed-address probing</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>ADR-007</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="35.15" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Phase gate</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Verified condition recorded in Phase_Gate_Status and Last_Verified_Gate that must PASS before a guided project enters the next lifecycle phase.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>DESIGN_GATE / PLAN_GATE / VERIFICATION_GATE</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>unverified phase jump</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>ADR-008</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="35.15" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Orchestration</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>State-machine selection of the next specialist skill by PROJECT-GUIDE using Current_Phase; never bypasses specialist rules or persistence gates.</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>guided delivery</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>automatic workflow execution</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>ADR-008</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35.15" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Focus mode</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Opt-in output-shaping mode from skill FOCUS-MODE: action-first, numbered steps, one concrete next step, lists capped at 5, no preamble or closers; never weakens sovereign rules, evidence labels or gate verdicts.</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>adhd mode</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>always-on output rewrite</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>ADR-009</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46.4" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Workbook mode</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Selected lifecycle operating context that determines the active workbook and behavior source.</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>HARNESS_MODE / PROJECT_MODE / MIGRATION_MODE</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>simultaneous default authorities</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>ADR-011</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="23.9" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Selected behavior source</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Single workbook from which the complete behavior catalog is read for the current mode.</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SELECTED_BEHAVIOR_SOURCE</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>concatenated duplicate catalogs</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>ADR-011</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35.15" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Routing oracle</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Frozen behavioral regression corpus in __ROUTING_ORACLE (L2 routing correctness, L3 adversarial/write-trap/SCRUB-completeness); out of the bootstrap read-set; run on explicit request or before promoting catalogue changes.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>__ROUTING_ORACLE / L2 corpus / L3 corpus</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>bootstrap read-set / silent auto-run</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>ADR-012</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="46.4" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Behavioral test</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>A model routing run against frozen Expected_Skill_ID and Expected_Verdict; distinct from a DETERMINISTIC_SCAN which only validates structure.</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>routing run / A/B routing test</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>self-report routing PASS</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>ADR-012</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35.15" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Status card</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory compact status block appended at the very end of replies after key events (bootstrap, guide steps, gates, revision commits, update context, explicit status): Mode, Resume, Gate, Verified (evidence-qualified only), Next.</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>status block</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>prose summary at reply start</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>ADR-013</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Allowed modes</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>00_Skills.Allowed_Modes value declaring in which workbook modes a skill may run: ALL or a comma-space separated subset of HARNESS, PROJECT, MIGRATION. Routing and CAPABILITY-DISCOVERY must not propose a skill outside the current mode.</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>mode allowlist</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>soft prose-based filtering</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>ADR-014</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="62.5" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Delivery schema</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Canonical definitions of the nine project delivery sheets (01_Plan..09_Worklog) embedded in sheet __DELIVERY_SCHEMA; PROJECT-FORK generates them into revision 001.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>__DELIVERY_SCHEMA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>physical project template</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ADR-017</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Starter sheet</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sheet _STARTER embedded in the kernel carrying the copilotstart contract; generated from copilot/copilotstart.txt at build time and read first on load vch. The repo txt remains the source of truth; blank lines are not preserved in the sheet.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>_STARTER</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>separate starter attachment</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ADR-019</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -579,7 +1378,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FROZEN ROUTING ORACLE v0.7.0 (out-of-bootstrap; L2 routing + L3 adversarial)</t>
+          <t>FROZEN ROUTING ORACLE v0.7.1 (out-of-bootstrap; L2 routing + L3 adversarial)</t>
         </is>
       </c>
     </row>
@@ -3551,7 +4350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3563,7 +4362,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>DELIVERY SCHEMA v0.7.0 (ADR-017; PROJECT-FORK generates these sheets into revision 001; out of the bootstrap read-set)</t>
+          <t>DELIVERY SCHEMA v0.7.1 (ADR-017; PROJECT-FORK generates these sheets into revision 001; out of the bootstrap read-set)</t>
         </is>
       </c>
     </row>
@@ -3753,6 +4552,610 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A94"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>####### Verifiable Copilot Harness - Copilot Starter v0.7.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Version v0.7.1  2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>This starter is embedded in the kernel workbook as the _STARTER sheet (ADR-019); attach only the workbook. The repo file copilot/copilotstart.txt is the source of truth and the lint asserts every non-empty sheet row matches it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Validate changed harness artifacts with harness_lint.ps1 before release promotion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>####### OPERATING MODEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Normal operation uses one active workbook:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>- VCH_HarnessCore.xlsx for non-project work and as the immutable project fork source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>- The current PROJECT_WORKBOOK to continue an existing project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Use multiple workbooks only for migration, lineage verification or explicit comparison. Select WORKBOOK_MODE before loading behavior. Read the complete behavior catalog once from SELECTED_BEHAVIOR_SOURCE. Never concatenate two catalogs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>####### WORKBOOK MODES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HARNESS_MODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- Active source: VCH_HarnessCore.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- Purpose: non-project work; immutable kernel and fork source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PROJECT_MODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Active source: the explicitly attached current PROJECT_WORKBOOK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- Use its embedded catalog as the behavior snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MIGRATION_MODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>- Inputs: old PROJECT_WORKBOOK plus current VCH_HarnessCore.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>- Keep the old project read-only and port verified project content only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>####### SOURCE SELECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>- Prefer an explicitly attached current project workbook for project continuation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>- Otherwise use VCH_HarnessCore.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>- Explicit binary attachments beat Work IQ results for editing and persistence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>- Multiple candidate current revisions return AMBIGUOUS_LINEAGE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>####### AUTHORITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SOVEREIGN SAFETY RULES outrank all lower layers: SCRUB, FROZEN ORACLE, EVIDENCE, NO CAPABILITY INHERITANCE and CHARACTER POLICY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Then: selected Project.Rules &gt; this starter &gt; selected 00_Skills &gt; selected __TEST_ORACLE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>A second attached workbook is not a second authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>####### ON "load vch"</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>- Select WORKBOOK_MODE and SELECTED_BEHAVIOR_SOURCE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>- Read _STARTER (this contract), Project.Rules, 00_Landing, __STATE, complete 00_Skills, __TEST_ORACLE, __ADR and __GLOSSARY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>- Do NOT read __ROUTING_ORACLE or __DELIVERY_SCHEMA on load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>- Run LOAD-ALL and BOOTSTRAP-CHECK read-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>- Report mode, behavior source, version, skill count, file role, goal, revision, lineage, Resume_From, Host_Mode, capability manifest and Persistence_Mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>- Missing persistence never blocks read-only work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>####### ROUTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Exact routing requires [skill: SKILL-ID] or a literal atomic Trigger. Trigger alternatives use exact ASCII " / ". May_Chain_To values use exact ASCII ", ". Otherwise apply Use_When, Do_Not_Use_When, Allowed_Modes and Precedence. Equal precedence uses lexicographically smallest Skill_ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>####### ALLOWED MODES</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>00_Skills.Allowed_Modes is either ALL or a canonical comma-space separated subset of HARNESS, PROJECT and MIGRATION. Never route or suggest a skill outside the current mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>####### ROUTING ORACLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>__ROUTING_ORACLE is a frozen out-of-bootstrap behavioral corpus with 55 fixtures: 43 L2 routing cases and 12 L3 adversarial cases. Never read or run it automatically. Run it only on explicit request or before catalog promotion. Structural lint validates schema and references only. Behavioral routing requires isolated execution against Expected_Skill_ID and Expected_Verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>####### DELIVERY SCHEMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>__DELIVERY_SCHEMA holds the canonical definitions of the nine project delivery sheets (01_Plan..09_Worklog). It is out of the bootstrap read-set. PROJECT-FORK reads it and generates the delivery sheets into revision 001; the kernel stays immutable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>####### HOST AND CAPABILITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Classify OPEN_WORKBOOK, ATTACHED_FILE, FILE_GROUNDING_ONLY or UNKNOWN separately from capability. Never inherit stored Capability_Mode as current runtime capability. Unknown capability remains UNTESTED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>####### PERSISTENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Persistent change routes through CAPABILITY-ROUTER:</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>- ARTIFACT_COPY_ON_WRITE after create, write, export, reopen and verify are proven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>- PRECOPIED_ARTIFACT for an exact verified SourceRevision+1 target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>- EXCEL_NATIVE_VERSIONING only in verified OPEN_WORKBOOK direct-edit mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>- Otherwise READ_ONLY or WRITE_BLOCKED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Never edit the immutable HarnessCore kernel for project delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>####### PROBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Probe only the __WRITE_PROBE value cell exposed as named range PROBE_CELL. Resolve by name, never by a fixed address. Use PRE-READ -&gt; WRITE UNIQUE TOKEN -&gt; READ-BACK -&gt; RESTORE ORIGINAL -&gt; FINAL READ-BACK and only on explicit request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>####### EVIDENCE AND OUTPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Classify evidence as INDEPENDENT_READ_BACK, TOOL_TRANSACTION_REPORT, CONVERSATION_EVIDENCE, SIMULATED_INPUT or INFERENCE. Self-report is not verification. Populate required fields or use UNKNOWN, NOT_PROVIDED, NOT_TESTED, NOT_APPLICABLE or PROPOSED_FIELD. SCRUB sensitive output before export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>####### STATUS CARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>After successful load, guide step, update context, phase gate, revision commit, explicit status request, or a change to Resume_From or Persistence_Mode, end with:</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Mode: {HARNESS|PROJECT|MIGRATION}</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Resume: {literal __STATE Resume_From value or none}</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Gate: {gate} -&gt; {PASS|BLOCKED|NOT_TESTED|n/a}</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Verified: {up to 3 INDEPENDENT_READ_BACK or TOOL_TRANSACTION_REPORT items}</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Next: {one concrete action} | Skill: {[skill: SKILL-ID] or none} | Why: {short clause}</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>The Status Card is the final block. It is not required for purely informational answers, SCRUB, focus toggling or routing oracle runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>####### NEXT FOOTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Every reply that does not end with a Status Card ends with exactly one final line:</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>NEXT: {one concrete action} ([skill: SKILL-ID])</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>or NEXT: none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>The recommended skill is only a May_Chain_To target of the skill just used, filtered by Allowed_Modes for the current mode. If May_Chain_To is NONE, propose update context in PROJECT mode, otherwise none. A recommendation is always a proposal; never chain automatically. The same exceptions as the Status Card apply: purely informational answers, SCRUB, focus toggling and routing oracle runs carry no footer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>####### FOCUS MODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Activate with "focus mode" or [skill: FOCUS-MODE]; deactivate with "focus mode off". First line is the next action, steps are bounded, lists are capped at 5 and each reply ends with one concrete next step (the NEXT footer or the Status Card Next line). Never remove evidence, gates or safety output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>####### RELEASE GATES</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>- STRUCTURAL_GATE: harness_lint.ps1 validates the kernel workbook, the _STARTER sheet against copilot/copilotstart.txt, the __DELIVERY_SCHEMA definitions and all implemented deterministic checks; a forked v001 must match __DELIVERY_SCHEMA exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>- BEHAVIORAL_ROUTING_GATE: execute all 55 routing rows in isolated contexts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>- Structural PASS never implies routing PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>- Any Critical=YES mismatch blocks catalog promotion.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3779,7 +5182,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SKILL CATALOGUE v0.7.0</t>
+          <t>SKILL CATALOGUE v0.7.1</t>
         </is>
       </c>
     </row>
@@ -3908,7 +5311,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -3983,7 +5386,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -4058,7 +5461,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -4133,7 +5536,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -4208,7 +5611,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -4283,7 +5686,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -4358,7 +5761,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -4433,7 +5836,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -4508,7 +5911,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -4583,7 +5986,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -4658,7 +6061,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -4733,7 +6136,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -4808,7 +6211,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -4883,7 +6286,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -4958,7 +6361,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -5033,7 +6436,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -5108,7 +6511,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -5183,7 +6586,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -5258,7 +6661,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -5333,7 +6736,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -5408,7 +6811,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -5483,7 +6886,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -5558,7 +6961,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -5633,7 +7036,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -5708,7 +7111,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -5783,7 +7186,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -5858,7 +7261,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -5933,7 +7336,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -6008,7 +7411,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -6083,7 +7486,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -6158,7 +7561,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -6233,7 +7636,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -6308,7 +7711,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -6383,7 +7786,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -6458,7 +7861,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -6533,7 +7936,7 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -6608,7 +8011,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -6683,7 +8086,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -6758,7 +8161,7 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -6833,7 +8236,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -6908,7 +8311,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -6983,7 +8386,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -7060,7 +8463,7 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -7095,7 +8498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7111,7 +8514,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PROJECT.RULES v0.7.0</t>
+          <t>PROJECT.RULES v0.7.1</t>
         </is>
       </c>
     </row>
@@ -7279,7 +8682,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>All components must agree on v0.7.0.</t>
+          <t>All components must agree on v0.7.1.</t>
         </is>
       </c>
     </row>
@@ -7387,7 +8790,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Use v0.7.0 for all harness and skill versions and NONE for an explicit empty canonical alternative. The strings None and none are forbidden as canonical tokens. Artifact_Status=REJECTED and Output_Verification_Status=OUTPUT_REJECTED are distinct field-scoped states.</t>
+          <t>Use v0.7.1 for all harness and skill versions and NONE for an explicit empty canonical alternative. The strings None and none are forbidden as canonical tokens. Artifact_Status=REJECTED and Output_Verification_Status=OUTPUT_REJECTED are distinct field-scoped states.</t>
         </is>
       </c>
     </row>
@@ -7517,7 +8920,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7533,7 +8936,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>__STATE v0.7.0</t>
+          <t>__STATE v0.7.1</t>
         </is>
       </c>
     </row>
@@ -7565,7 +8968,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
     </row>
@@ -7589,7 +8992,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
     </row>
@@ -7721,7 +9124,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>VCH_HarnessCore.xlsx v6.15.1</t>
+          <t>VCH_HarnessCore.xlsx v0.7.0</t>
         </is>
       </c>
     </row>
@@ -7949,7 +9352,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>VCH_HarnessCore.xlsx v6.15.1; ADR-018</t>
+          <t>VCH_HarnessCore.xlsx v0.7.0; ADR-019</t>
         </is>
       </c>
     </row>
@@ -8019,7 +9422,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8035,7 +9438,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>00 Landing v0.7.0</t>
+          <t>00 Landing v0.7.1</t>
         </is>
       </c>
     </row>
@@ -8182,7 +9585,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
     </row>
@@ -8384,13 +9787,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8405,7 +9808,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FROZEN TEST ORACLE v0.7.0</t>
+          <t>FROZEN TEST ORACLE v0.7.1</t>
         </is>
       </c>
     </row>
@@ -8803,7 +10206,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -8828,7 +10231,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>All version fields across sheets agree on v0.7.0.</t>
+          <t>All version fields across sheets agree on v0.7.1.</t>
         </is>
       </c>
     </row>
@@ -8850,7 +10253,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>v0.7.0</t>
+          <t>v0.7.1</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -8875,7 +10278,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>All 43 skill rows use canonical v0.7.0.</t>
+          <t>All 43 skill rows use canonical v0.7.1.</t>
         </is>
       </c>
     </row>
@@ -9722,6 +11125,53 @@
       <c r="I29" t="inlineStr">
         <is>
           <t>__DELIVERY_SCHEMA exists with all 9 delivery sheet definitions; a forked v001 matches them exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>STARTER</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Starter_Sheet_Present</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>DETERMINISTIC_SCAN</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>_STARTER sheet exists and every non-empty row reproduces copilotstart.txt line-for-line; harness_lint compares the sheet against the repo file.</t>
         </is>
       </c>
     </row>
@@ -9731,7 +11181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9746,7 +11196,7 @@
     <row r="1" ht="15.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CANONICAL LISTS v0.7.0</t>
+          <t>CANONICAL LISTS v0.7.1</t>
         </is>
       </c>
     </row>
@@ -10439,13 +11889,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11297,769 +12747,55 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.5" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PROJECT GLOSSARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Aliases</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Do_Not_Use</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Updated</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Host mode</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Workbook interaction context independent from capability.</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>OPEN_WORKBOOK</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>write capability</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>ADR-004</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Precopied artifact</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>User-created canonical next revision verified before activation.</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Save a Copy target</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>storage suffix copy</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ADR-004</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Logical checkpoint</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Verified in-place state change with no new physical artifact.</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>native revision</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>physical revision</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>ADR-004</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="23.9" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Trigger delimiter</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>ASCII sequence " / " separating alternative literal triggers only in 00_Skills.Trigger.</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>slash-delimited aliases</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>global slash splitting</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="23.9" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Chain delimiter</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>ASCII sequence ", " separating Skill_ID values only in 00_Skills.May_Chain_To.</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>comma-delimited chain</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>global comma splitting</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Field-scoped enum</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Canonical enum value interpreted together with its field name.</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Field=Value</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>unqualified status token</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="23.9" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Output rejected</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Output verification state OUTPUT_REJECTED; distinct from Artifact_Status=REJECTED.</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>OUTPUT_REJECTED</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>artifact rejected</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="23.9" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Artifact rejected</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Artifact lifecycle state REJECTED; distinct from Output_Verification_Status=OUTPUT_REJECTED.</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>output rejected</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Canonical NONE</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Explicit empty canonical alternative represented by ASCII token NONE.</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>None / none</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="35.15" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Sovereign rules</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Safety rules that no lower authority layer may weaken: SCRUB, FROZEN ORACLE, EVIDENCE, NO CAPABILITY INHERITANCE, CHARACTER POLICY.</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>authority layer 0</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>overridable safety</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>ADR-007</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="23.9" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Version migration</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Controlled port of an older-version workbook into a new revision forked from the current kernel after a VERSION_MISMATCH report.</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>kernel upgrade</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>silent rewrite</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>ADR-007</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="35.15" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Probe cell</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Value cell of the __WRITE_PROBE field in __STATE, exposed as named range PROBE_CELL (currently __STATE!B31); the only legal direct-edit probe target, always resolved by name.</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>PROBE_CELL</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>fixed-address probing</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>ADR-007</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="35.15" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Phase gate</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Verified condition recorded in Phase_Gate_Status and Last_Verified_Gate that must PASS before a guided project enters the next lifecycle phase.</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>DESIGN_GATE / PLAN_GATE / VERIFICATION_GATE</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>unverified phase jump</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>ADR-008</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="35.15" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Orchestration</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>State-machine selection of the next specialist skill by PROJECT-GUIDE using Current_Phase; never bypasses specialist rules or persistence gates.</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>guided delivery</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>automatic workflow execution</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>ADR-008</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="35.15" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Focus mode</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Opt-in output-shaping mode from skill FOCUS-MODE: action-first, numbered steps, one concrete next step, lists capped at 5, no preamble or closers; never weakens sovereign rules, evidence labels or gate verdicts.</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>adhd mode</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>always-on output rewrite</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>ADR-009</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="46.4" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Workbook mode</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Selected lifecycle operating context that determines the active workbook and behavior source.</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>HARNESS_MODE / PROJECT_MODE / MIGRATION_MODE</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>simultaneous default authorities</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>ADR-011</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="23.9" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Selected behavior source</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Single workbook from which the complete behavior catalog is read for the current mode.</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>SELECTED_BEHAVIOR_SOURCE</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>concatenated duplicate catalogs</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>ADR-011</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="35.15" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Routing oracle</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Frozen behavioral regression corpus in __ROUTING_ORACLE (L2 routing correctness, L3 adversarial/write-trap/SCRUB-completeness); out of the bootstrap read-set; run on explicit request or before promoting catalogue changes.</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>__ROUTING_ORACLE / L2 corpus / L3 corpus</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>bootstrap read-set / silent auto-run</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>ADR-012</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="46.4" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Behavioral test</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>A model routing run against frozen Expected_Skill_ID and Expected_Verdict; distinct from a DETERMINISTIC_SCAN which only validates structure.</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>routing run / A/B routing test</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>self-report routing PASS</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>ADR-012</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="35.15" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Status card</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Mandatory compact status block appended at the very end of replies after key events (bootstrap, guide steps, gates, revision commits, update context, explicit status): Mode, Resume, Gate, Verified (evidence-qualified only), Next.</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>status block</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>prose summary at reply start</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>ADR-013</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="50" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Allowed modes</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>00_Skills.Allowed_Modes value declaring in which workbook modes a skill may run: ALL or a comma-space separated subset of HARNESS, PROJECT, MIGRATION. Routing and CAPABILITY-DISCOVERY must not propose a skill outside the current mode.</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>mode allowlist</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>soft prose-based filtering</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>ADR-014</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="62.5" customHeight="1">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Delivery schema</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Canonical definitions of the nine project delivery sheets (01_Plan..09_Worklog) embedded in sheet __DELIVERY_SCHEMA; PROJECT-FORK generates them into revision 001.</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>__DELIVERY_SCHEMA</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>physical project template</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>ADR-017</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ADR-019</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Embed copilotstart.txt as the _STARTER sheet in the kernel; the txt stays the repo source of truth and the lint asserts every non-empty sheet row equals the file line</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>After ADR-017 the starter was the only behavior text outside the artifact. Version drift between the attached starter and the kernel was unverifiable at runtime, and two attachments per session were the last avoidable onboarding step.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Keep a separate starter txt; embed a generated _STARTER sheet; embed and delete the txt from the repo.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>A version-locked artifact removes starter/kernel drift by construction, the same argument as ADR-012 for the routing oracle. Keeping the txt as the build source preserves git-diffable review; the sheet is generated, never hand-edited.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Attach flow becomes one workbook per session; custom instructions start the bootstrap read-set with _STARTER; harness_lint gains the STARTER sheet-versus-file check; __TEST_ORACLE gains Starter_Sheet_Present; copilot_custom_instructions.txt stays outside because it configures Copilot itself and cannot be attached. All components bump to v0.7.1.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Delete the _STARTER sheet and attach copilot/copilotstart.txt again; the txt is kept in the repo unchanged in role.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Owner request 2026-07-27; tools/build_v071.py.</t>
         </is>
       </c>
     </row>

</xml_diff>